<commit_message>
Add webapp UI for Sudoku solver and deployment assets
</commit_message>
<xml_diff>
--- a/results/conference_results.xlsx
+++ b/results/conference_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Thesis\Progress\Original Repo\Multi swarm\ACS-SA-RING\MT-ACS-RING\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8701F07-92C0-4C8E-966C-1ADA4EC01BC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1500142-EE63-478A-B203-83AFE3EE5E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0FB7F815-C557-4D5B-A7D0-2D04B3DEB5B3}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{0FB7F815-C557-4D5B-A7D0-2D04B3DEB5B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="50">
   <si>
     <t>Size</t>
   </si>
@@ -415,12 +415,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -458,6 +455,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -479,7 +479,16 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -816,14 +825,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9221DC26-A763-4BCD-9281-6B369DCA2C66}">
-  <dimension ref="B2:S63"/>
+  <dimension ref="B2:U63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="7.42578125" customWidth="1"/>
     <col min="3" max="3" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B2" s="22" t="s">
         <v>0</v>
       </c>
@@ -848,129 +857,132 @@
       <c r="M2" s="28"/>
       <c r="N2" s="28"/>
       <c r="O2" s="28"/>
-      <c r="P2" s="29" t="s">
+      <c r="P2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="Q2" s="29"/>
-      <c r="R2" s="29"/>
-      <c r="S2" s="29"/>
-    </row>
-    <row r="3" spans="2:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="S2" s="21"/>
+    </row>
+    <row r="3" spans="2:21" ht="30" x14ac:dyDescent="0.25">
       <c r="B3" s="23"/>
       <c r="C3" s="25"/>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="L3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="M3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="N3" s="7" t="s">
+      <c r="N3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="O3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="P3" s="8" t="s">
+      <c r="P3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="Q3" s="8" t="s">
+      <c r="Q3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="R3" s="8" t="s">
+      <c r="R3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="S3" s="8" t="s">
+      <c r="S3" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B4" s="9">
+    <row r="4" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B4" s="8">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>99</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="9">
         <v>9.1009999999999994E-2</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="9">
         <v>0.49808000000000002</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="10">
         <v>178.91</v>
       </c>
-      <c r="H4" s="9">
-        <v>100</v>
-      </c>
-      <c r="I4" s="10">
+      <c r="H4" s="8">
+        <v>100</v>
+      </c>
+      <c r="I4" s="9">
         <v>4.7039999999999998E-2</v>
       </c>
-      <c r="J4" s="10">
+      <c r="J4" s="9">
         <v>4.6059999999999997E-2</v>
       </c>
-      <c r="K4" s="10">
+      <c r="K4" s="9">
         <v>64.13</v>
       </c>
-      <c r="L4" s="9">
-        <v>100</v>
-      </c>
-      <c r="M4" s="10">
+      <c r="L4" s="8">
+        <v>100</v>
+      </c>
+      <c r="M4" s="9">
         <v>1.6629999999999999E-2</v>
       </c>
-      <c r="N4" s="10">
+      <c r="N4" s="9">
         <v>1.384E-2</v>
       </c>
-      <c r="O4" s="11">
+      <c r="O4" s="10">
         <v>24.04</v>
       </c>
-      <c r="P4" s="9">
-        <v>100</v>
-      </c>
-      <c r="Q4" s="10">
+      <c r="P4" s="8">
+        <v>100</v>
+      </c>
+      <c r="Q4" s="9">
         <v>2.733E-2</v>
       </c>
-      <c r="R4" s="10">
+      <c r="R4" s="9">
         <v>2.8230000000000002E-2</v>
       </c>
-      <c r="S4" s="11">
+      <c r="S4" s="10">
         <v>25.32</v>
       </c>
-    </row>
-    <row r="5" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="12">
+      <c r="U4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B5" s="11">
         <v>3</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="11">
         <v>99</v>
       </c>
       <c r="E5">
@@ -979,10 +991,10 @@
       <c r="F5">
         <v>7.9680000000000001E-2</v>
       </c>
-      <c r="G5" s="14">
+      <c r="G5" s="13">
         <v>109.98</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="11">
         <v>100</v>
       </c>
       <c r="I5">
@@ -994,7 +1006,7 @@
       <c r="K5">
         <v>94.07</v>
       </c>
-      <c r="L5" s="12">
+      <c r="L5" s="11">
         <v>100</v>
       </c>
       <c r="M5">
@@ -1003,10 +1015,10 @@
       <c r="N5">
         <v>2.7390000000000001E-2</v>
       </c>
-      <c r="O5" s="14">
+      <c r="O5" s="13">
         <v>27.43</v>
       </c>
-      <c r="P5" s="12">
+      <c r="P5" s="11">
         <v>100</v>
       </c>
       <c r="Q5">
@@ -1015,18 +1027,21 @@
       <c r="R5">
         <v>7.6399999999999996E-2</v>
       </c>
-      <c r="S5" s="14">
+      <c r="S5" s="13">
         <v>33.119999999999997</v>
       </c>
-    </row>
-    <row r="6" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B6" s="12">
+      <c r="U5" s="12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B6" s="11">
         <v>3</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="11">
         <v>99</v>
       </c>
       <c r="E6">
@@ -1035,10 +1050,10 @@
       <c r="F6">
         <v>0.10705000000000001</v>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="13">
         <v>187.62</v>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="11">
         <v>100</v>
       </c>
       <c r="I6">
@@ -1050,7 +1065,7 @@
       <c r="K6">
         <v>207</v>
       </c>
-      <c r="L6" s="12">
+      <c r="L6" s="11">
         <v>100</v>
       </c>
       <c r="M6">
@@ -1059,10 +1074,10 @@
       <c r="N6">
         <v>6.8970000000000004E-2</v>
       </c>
-      <c r="O6" s="14">
+      <c r="O6" s="13">
         <v>71.58</v>
       </c>
-      <c r="P6" s="12">
+      <c r="P6" s="11">
         <v>100</v>
       </c>
       <c r="Q6">
@@ -1071,18 +1086,21 @@
       <c r="R6">
         <v>0.12229</v>
       </c>
-      <c r="S6" s="14">
+      <c r="S6" s="13">
         <v>70.849999999999994</v>
       </c>
-    </row>
-    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B7" s="12">
+      <c r="U6" s="12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B7" s="11">
         <v>3</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="11">
         <v>100</v>
       </c>
       <c r="E7">
@@ -1091,10 +1109,10 @@
       <c r="F7">
         <v>4.9279999999999997E-2</v>
       </c>
-      <c r="G7" s="14">
+      <c r="G7" s="13">
         <v>87.96</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="11">
         <v>100</v>
       </c>
       <c r="I7">
@@ -1106,7 +1124,7 @@
       <c r="K7">
         <v>88.58</v>
       </c>
-      <c r="L7" s="12">
+      <c r="L7" s="11">
         <v>100</v>
       </c>
       <c r="M7">
@@ -1115,10 +1133,10 @@
       <c r="N7">
         <v>2.0809999999999999E-2</v>
       </c>
-      <c r="O7" s="14">
+      <c r="O7" s="13">
         <v>32.76</v>
       </c>
-      <c r="P7" s="12">
+      <c r="P7" s="11">
         <v>100</v>
       </c>
       <c r="Q7">
@@ -1127,18 +1145,21 @@
       <c r="R7">
         <v>5.4859999999999999E-2</v>
       </c>
-      <c r="S7" s="14">
+      <c r="S7" s="13">
         <v>35.19</v>
       </c>
-    </row>
-    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B8" s="12">
+      <c r="U7" s="12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B8" s="11">
         <v>3</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="11">
         <v>100</v>
       </c>
       <c r="E8">
@@ -1147,10 +1168,10 @@
       <c r="F8">
         <v>6.4820000000000003E-2</v>
       </c>
-      <c r="G8" s="14">
+      <c r="G8" s="13">
         <v>95.11</v>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="11">
         <v>100</v>
       </c>
       <c r="I8">
@@ -1162,7 +1183,7 @@
       <c r="K8">
         <v>90.88</v>
       </c>
-      <c r="L8" s="12">
+      <c r="L8" s="11">
         <v>100</v>
       </c>
       <c r="M8">
@@ -1171,10 +1192,10 @@
       <c r="N8">
         <v>3.2250000000000001E-2</v>
       </c>
-      <c r="O8" s="14">
+      <c r="O8" s="13">
         <v>26.14</v>
       </c>
-      <c r="P8" s="12">
+      <c r="P8" s="11">
         <v>100</v>
       </c>
       <c r="Q8">
@@ -1183,18 +1204,21 @@
       <c r="R8">
         <v>3.9550000000000002E-2</v>
       </c>
-      <c r="S8" s="14">
+      <c r="S8" s="13">
         <v>29.21</v>
       </c>
-    </row>
-    <row r="9" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="12">
+      <c r="U8" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B9" s="11">
         <v>3</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="11">
         <v>100</v>
       </c>
       <c r="E9">
@@ -1203,10 +1227,10 @@
       <c r="F9">
         <v>8.548E-2</v>
       </c>
-      <c r="G9" s="14">
+      <c r="G9" s="13">
         <v>109.87</v>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="11">
         <v>100</v>
       </c>
       <c r="I9">
@@ -1218,7 +1242,7 @@
       <c r="K9">
         <v>108.47</v>
       </c>
-      <c r="L9" s="12">
+      <c r="L9" s="11">
         <v>100</v>
       </c>
       <c r="M9">
@@ -1227,10 +1251,10 @@
       <c r="N9">
         <v>2.2960000000000001E-2</v>
       </c>
-      <c r="O9" s="14">
+      <c r="O9" s="13">
         <v>30.85</v>
       </c>
-      <c r="P9" s="12">
+      <c r="P9" s="11">
         <v>100</v>
       </c>
       <c r="Q9">
@@ -1239,18 +1263,21 @@
       <c r="R9">
         <v>5.2490000000000002E-2</v>
       </c>
-      <c r="S9" s="14">
+      <c r="S9" s="13">
         <v>33.07</v>
       </c>
-    </row>
-    <row r="10" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="12">
+      <c r="U9" s="12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B10" s="11">
         <v>3</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="11">
         <v>100</v>
       </c>
       <c r="E10">
@@ -1259,10 +1286,10 @@
       <c r="F10">
         <v>4.8379999999999999E-2</v>
       </c>
-      <c r="G10" s="14">
+      <c r="G10" s="13">
         <v>90.94</v>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="11">
         <v>100</v>
       </c>
       <c r="I10">
@@ -1274,7 +1301,7 @@
       <c r="K10">
         <v>79.41</v>
       </c>
-      <c r="L10" s="12">
+      <c r="L10" s="11">
         <v>100</v>
       </c>
       <c r="M10">
@@ -1283,10 +1310,10 @@
       <c r="N10">
         <v>1.9740000000000001E-2</v>
       </c>
-      <c r="O10" s="14">
+      <c r="O10" s="13">
         <v>34.72</v>
       </c>
-      <c r="P10" s="12">
+      <c r="P10" s="11">
         <v>100</v>
       </c>
       <c r="Q10">
@@ -1295,18 +1322,21 @@
       <c r="R10">
         <v>3.6409999999999998E-2</v>
       </c>
-      <c r="S10" s="14">
+      <c r="S10" s="13">
         <v>33.200000000000003</v>
       </c>
-    </row>
-    <row r="11" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="12">
+      <c r="U10" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B11" s="11">
         <v>3</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="11">
         <v>100</v>
       </c>
       <c r="E11">
@@ -1315,10 +1345,10 @@
       <c r="F11">
         <v>2.9239999999999999E-2</v>
       </c>
-      <c r="G11" s="14">
+      <c r="G11" s="13">
         <v>50.53</v>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="11">
         <v>100</v>
       </c>
       <c r="I11">
@@ -1330,7 +1360,7 @@
       <c r="K11">
         <v>52.5</v>
       </c>
-      <c r="L11" s="12">
+      <c r="L11" s="11">
         <v>100</v>
       </c>
       <c r="M11">
@@ -1339,10 +1369,10 @@
       <c r="N11">
         <v>1.103E-2</v>
       </c>
-      <c r="O11" s="14">
+      <c r="O11" s="13">
         <v>15.42</v>
       </c>
-      <c r="P11" s="12">
+      <c r="P11" s="11">
         <v>100</v>
       </c>
       <c r="Q11">
@@ -1351,18 +1381,21 @@
       <c r="R11">
         <v>1.7049999999999999E-2</v>
       </c>
-      <c r="S11" s="14">
+      <c r="S11" s="13">
         <v>17.760000000000002</v>
       </c>
-    </row>
-    <row r="12" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B12" s="12">
+      <c r="U11" s="12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B12" s="11">
         <v>3</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="11">
         <v>100</v>
       </c>
       <c r="E12">
@@ -1371,10 +1404,10 @@
       <c r="F12">
         <v>8.5680000000000006E-2</v>
       </c>
-      <c r="G12" s="14">
+      <c r="G12" s="13">
         <v>116.63</v>
       </c>
-      <c r="H12" s="12">
+      <c r="H12" s="11">
         <v>100</v>
       </c>
       <c r="I12">
@@ -1386,7 +1419,7 @@
       <c r="K12">
         <v>116.79</v>
       </c>
-      <c r="L12" s="12">
+      <c r="L12" s="11">
         <v>100</v>
       </c>
       <c r="M12">
@@ -1395,10 +1428,10 @@
       <c r="N12">
         <v>2.4559999999999998E-2</v>
       </c>
-      <c r="O12" s="14">
+      <c r="O12" s="13">
         <v>40.58</v>
       </c>
-      <c r="P12" s="12">
+      <c r="P12" s="11">
         <v>100</v>
       </c>
       <c r="Q12">
@@ -1407,18 +1440,21 @@
       <c r="R12">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="S12" s="14">
+      <c r="S12" s="13">
         <v>49.07</v>
       </c>
-    </row>
-    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B13" s="12">
+      <c r="U12" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B13" s="11">
         <v>3</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="11">
         <v>100</v>
       </c>
       <c r="E13">
@@ -1427,10 +1463,10 @@
       <c r="F13">
         <v>9.98E-2</v>
       </c>
-      <c r="G13" s="14">
+      <c r="G13" s="13">
         <v>110.81</v>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="11">
         <v>100</v>
       </c>
       <c r="I13">
@@ -1442,7 +1478,7 @@
       <c r="K13">
         <v>107.71</v>
       </c>
-      <c r="L13" s="12">
+      <c r="L13" s="11">
         <v>100</v>
       </c>
       <c r="M13">
@@ -1451,10 +1487,10 @@
       <c r="N13">
         <v>2.291E-2</v>
       </c>
-      <c r="O13" s="14">
+      <c r="O13" s="13">
         <v>38.92</v>
       </c>
-      <c r="P13" s="12">
+      <c r="P13" s="11">
         <v>100</v>
       </c>
       <c r="Q13">
@@ -1463,18 +1499,21 @@
       <c r="R13">
         <v>5.6320000000000002E-2</v>
       </c>
-      <c r="S13" s="14">
+      <c r="S13" s="13">
         <v>34.630000000000003</v>
       </c>
-    </row>
-    <row r="14" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="12">
+      <c r="U13" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B14" s="11">
         <v>3</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="11">
         <v>100</v>
       </c>
       <c r="E14">
@@ -1483,10 +1522,10 @@
       <c r="F14">
         <v>9.6790000000000001E-2</v>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="13">
         <v>167.01</v>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="11">
         <v>100</v>
       </c>
       <c r="I14">
@@ -1498,7 +1537,7 @@
       <c r="K14">
         <v>139.35</v>
       </c>
-      <c r="L14" s="12">
+      <c r="L14" s="11">
         <v>100</v>
       </c>
       <c r="M14">
@@ -1507,10 +1546,10 @@
       <c r="N14">
         <v>2.0480000000000002E-2</v>
       </c>
-      <c r="O14" s="14">
+      <c r="O14" s="13">
         <v>39.14</v>
       </c>
-      <c r="P14" s="12">
+      <c r="P14" s="11">
         <v>100</v>
       </c>
       <c r="Q14">
@@ -1519,18 +1558,18 @@
       <c r="R14">
         <v>5.8450000000000002E-2</v>
       </c>
-      <c r="S14" s="14">
+      <c r="S14" s="13">
         <v>41.28</v>
       </c>
     </row>
-    <row r="15" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B15" s="12">
+    <row r="15" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B15" s="11">
         <v>3</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="11">
         <v>100</v>
       </c>
       <c r="E15">
@@ -1539,10 +1578,10 @@
       <c r="F15">
         <v>6.5079999999999999E-2</v>
       </c>
-      <c r="G15" s="14">
+      <c r="G15" s="13">
         <v>108.49</v>
       </c>
-      <c r="H15" s="12">
+      <c r="H15" s="11">
         <v>100</v>
       </c>
       <c r="I15">
@@ -1554,7 +1593,7 @@
       <c r="K15">
         <v>106.58</v>
       </c>
-      <c r="L15" s="12">
+      <c r="L15" s="11">
         <v>100</v>
       </c>
       <c r="M15">
@@ -1563,10 +1602,10 @@
       <c r="N15">
         <v>2.0500000000000001E-2</v>
       </c>
-      <c r="O15" s="14">
+      <c r="O15" s="13">
         <v>36.659999999999997</v>
       </c>
-      <c r="P15" s="12">
+      <c r="P15" s="11">
         <v>100</v>
       </c>
       <c r="Q15">
@@ -1575,18 +1614,18 @@
       <c r="R15">
         <v>4.4889999999999999E-2</v>
       </c>
-      <c r="S15" s="14">
+      <c r="S15" s="13">
         <v>32.1</v>
       </c>
     </row>
-    <row r="16" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B16" s="12">
+    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B16" s="11">
         <v>3</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="11">
         <v>100</v>
       </c>
       <c r="E16">
@@ -1595,10 +1634,10 @@
       <c r="F16">
         <v>4.929E-2</v>
       </c>
-      <c r="G16" s="14">
+      <c r="G16" s="13">
         <v>78.34</v>
       </c>
-      <c r="H16" s="12">
+      <c r="H16" s="11">
         <v>100</v>
       </c>
       <c r="I16">
@@ -1610,7 +1649,7 @@
       <c r="K16">
         <v>80.739999999999995</v>
       </c>
-      <c r="L16" s="12">
+      <c r="L16" s="11">
         <v>100</v>
       </c>
       <c r="M16">
@@ -1619,10 +1658,10 @@
       <c r="N16">
         <v>1.617E-2</v>
       </c>
-      <c r="O16" s="14">
+      <c r="O16" s="13">
         <v>27.48</v>
       </c>
-      <c r="P16" s="12">
+      <c r="P16" s="11">
         <v>100</v>
       </c>
       <c r="Q16">
@@ -1631,18 +1670,18 @@
       <c r="R16">
         <v>3.2039999999999999E-2</v>
       </c>
-      <c r="S16" s="14">
+      <c r="S16" s="13">
         <v>25.19</v>
       </c>
     </row>
     <row r="17" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="12">
+      <c r="B17" s="11">
         <v>3</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="12">
+      <c r="D17" s="11">
         <v>100</v>
       </c>
       <c r="E17">
@@ -1651,10 +1690,10 @@
       <c r="F17">
         <v>8.0339999999999995E-2</v>
       </c>
-      <c r="G17" s="14">
+      <c r="G17" s="13">
         <v>122.24</v>
       </c>
-      <c r="H17" s="12">
+      <c r="H17" s="11">
         <v>100</v>
       </c>
       <c r="I17">
@@ -1666,7 +1705,7 @@
       <c r="K17">
         <v>109.84</v>
       </c>
-      <c r="L17" s="12">
+      <c r="L17" s="11">
         <v>100</v>
       </c>
       <c r="M17">
@@ -1675,10 +1714,10 @@
       <c r="N17">
         <v>2.5989999999999999E-2</v>
       </c>
-      <c r="O17" s="14">
+      <c r="O17" s="13">
         <v>41.55</v>
       </c>
-      <c r="P17" s="12">
+      <c r="P17" s="11">
         <v>100</v>
       </c>
       <c r="Q17">
@@ -1687,18 +1726,18 @@
       <c r="R17">
         <v>6.2530000000000002E-2</v>
       </c>
-      <c r="S17" s="14">
+      <c r="S17" s="13">
         <v>46.1</v>
       </c>
     </row>
     <row r="18" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B18" s="12">
+      <c r="B18" s="11">
         <v>3</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="11">
         <v>100</v>
       </c>
       <c r="E18">
@@ -1707,10 +1746,10 @@
       <c r="F18">
         <v>5.9479999999999998E-2</v>
       </c>
-      <c r="G18" s="14">
+      <c r="G18" s="13">
         <v>104.05</v>
       </c>
-      <c r="H18" s="12">
+      <c r="H18" s="11">
         <v>100</v>
       </c>
       <c r="I18">
@@ -1722,7 +1761,7 @@
       <c r="K18">
         <v>94.66</v>
       </c>
-      <c r="L18" s="12">
+      <c r="L18" s="11">
         <v>100</v>
       </c>
       <c r="M18">
@@ -1731,10 +1770,10 @@
       <c r="N18">
         <v>2.5020000000000001E-2</v>
       </c>
-      <c r="O18" s="14">
+      <c r="O18" s="13">
         <v>36.01</v>
       </c>
-      <c r="P18" s="12">
+      <c r="P18" s="11">
         <v>100</v>
       </c>
       <c r="Q18">
@@ -1743,18 +1782,18 @@
       <c r="R18">
         <v>4.8820000000000002E-2</v>
       </c>
-      <c r="S18" s="14">
+      <c r="S18" s="13">
         <v>34.840000000000003</v>
       </c>
     </row>
     <row r="19" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B19" s="12">
+      <c r="B19" s="11">
         <v>3</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="11">
         <v>100</v>
       </c>
       <c r="E19">
@@ -1763,10 +1802,10 @@
       <c r="F19">
         <v>6.9739999999999996E-2</v>
       </c>
-      <c r="G19" s="14">
+      <c r="G19" s="13">
         <v>105.52</v>
       </c>
-      <c r="H19" s="12">
+      <c r="H19" s="11">
         <v>100</v>
       </c>
       <c r="I19">
@@ -1778,7 +1817,7 @@
       <c r="K19">
         <v>95.2</v>
       </c>
-      <c r="L19" s="12">
+      <c r="L19" s="11">
         <v>100</v>
       </c>
       <c r="M19">
@@ -1787,10 +1826,10 @@
       <c r="N19">
         <v>3.0880000000000001E-2</v>
       </c>
-      <c r="O19" s="14">
+      <c r="O19" s="13">
         <v>34.799999999999997</v>
       </c>
-      <c r="P19" s="12">
+      <c r="P19" s="11">
         <v>100</v>
       </c>
       <c r="Q19">
@@ -1799,18 +1838,18 @@
       <c r="R19">
         <v>5.2769999999999997E-2</v>
       </c>
-      <c r="S19" s="14">
+      <c r="S19" s="13">
         <v>30.81</v>
       </c>
     </row>
     <row r="20" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B20" s="12">
+      <c r="B20" s="11">
         <v>3</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="11">
         <v>100</v>
       </c>
       <c r="E20">
@@ -1819,10 +1858,10 @@
       <c r="F20">
         <v>6.5460000000000004E-2</v>
       </c>
-      <c r="G20" s="14">
+      <c r="G20" s="13">
         <v>115.91</v>
       </c>
-      <c r="H20" s="12">
+      <c r="H20" s="11">
         <v>100</v>
       </c>
       <c r="I20">
@@ -1834,7 +1873,7 @@
       <c r="K20">
         <v>101.14</v>
       </c>
-      <c r="L20" s="12">
+      <c r="L20" s="11">
         <v>100</v>
       </c>
       <c r="M20">
@@ -1843,10 +1882,10 @@
       <c r="N20">
         <v>3.5479999999999998E-2</v>
       </c>
-      <c r="O20" s="14">
+      <c r="O20" s="13">
         <v>36.46</v>
       </c>
-      <c r="P20" s="12">
+      <c r="P20" s="11">
         <v>100</v>
       </c>
       <c r="Q20">
@@ -1855,18 +1894,18 @@
       <c r="R20">
         <v>5.5980000000000002E-2</v>
       </c>
-      <c r="S20" s="14">
+      <c r="S20" s="13">
         <v>36.69</v>
       </c>
     </row>
     <row r="21" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B21" s="12">
+      <c r="B21" s="11">
         <v>3</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="11">
         <v>100</v>
       </c>
       <c r="E21">
@@ -1875,10 +1914,10 @@
       <c r="F21">
         <v>4.7739999999999998E-2</v>
       </c>
-      <c r="G21" s="14">
+      <c r="G21" s="13">
         <v>92.03</v>
       </c>
-      <c r="H21" s="12">
+      <c r="H21" s="11">
         <v>100</v>
       </c>
       <c r="I21">
@@ -1890,7 +1929,7 @@
       <c r="K21">
         <v>93.69</v>
       </c>
-      <c r="L21" s="12">
+      <c r="L21" s="11">
         <v>100</v>
       </c>
       <c r="M21">
@@ -1899,10 +1938,10 @@
       <c r="N21">
         <v>1.951E-2</v>
       </c>
-      <c r="O21" s="14">
+      <c r="O21" s="13">
         <v>29.89</v>
       </c>
-      <c r="P21" s="12">
+      <c r="P21" s="11">
         <v>100</v>
       </c>
       <c r="Q21">
@@ -1911,18 +1950,18 @@
       <c r="R21">
         <v>3.7080000000000002E-2</v>
       </c>
-      <c r="S21" s="14">
+      <c r="S21" s="13">
         <v>31.91</v>
       </c>
     </row>
     <row r="22" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B22" s="12">
+      <c r="B22" s="11">
         <v>3</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="11">
         <v>100</v>
       </c>
       <c r="E22">
@@ -1931,10 +1970,10 @@
       <c r="F22">
         <v>6.4019999999999994E-2</v>
       </c>
-      <c r="G22" s="14">
+      <c r="G22" s="13">
         <v>102.46</v>
       </c>
-      <c r="H22" s="12">
+      <c r="H22" s="11">
         <v>100</v>
       </c>
       <c r="I22">
@@ -1946,7 +1985,7 @@
       <c r="K22">
         <v>109.36</v>
       </c>
-      <c r="L22" s="12">
+      <c r="L22" s="11">
         <v>100</v>
       </c>
       <c r="M22">
@@ -1955,10 +1994,10 @@
       <c r="N22">
         <v>4.7190000000000003E-2</v>
       </c>
-      <c r="O22" s="14">
+      <c r="O22" s="13">
         <v>35.229999999999997</v>
       </c>
-      <c r="P22" s="12">
+      <c r="P22" s="11">
         <v>100</v>
       </c>
       <c r="Q22">
@@ -1967,130 +2006,130 @@
       <c r="R22">
         <v>5.552E-2</v>
       </c>
-      <c r="S22" s="14">
+      <c r="S22" s="13">
         <v>41.58</v>
       </c>
     </row>
     <row r="23" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B23" s="15">
+      <c r="B23" s="14">
         <v>3</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="15">
-        <v>100</v>
-      </c>
-      <c r="E23" s="16">
+      <c r="D23" s="14">
+        <v>100</v>
+      </c>
+      <c r="E23" s="15">
         <v>0.14465</v>
       </c>
-      <c r="F23" s="16">
+      <c r="F23" s="15">
         <v>0.14660999999999999</v>
       </c>
-      <c r="G23" s="17">
+      <c r="G23" s="16">
         <v>205.1</v>
       </c>
-      <c r="H23" s="15">
-        <v>100</v>
-      </c>
-      <c r="I23" s="16">
+      <c r="H23" s="14">
+        <v>100</v>
+      </c>
+      <c r="I23" s="15">
         <v>0.27088000000000001</v>
       </c>
-      <c r="J23" s="16">
+      <c r="J23" s="15">
         <v>0.38075999999999999</v>
       </c>
-      <c r="K23" s="16">
+      <c r="K23" s="15">
         <v>205.41</v>
       </c>
-      <c r="L23" s="15">
-        <v>100</v>
-      </c>
-      <c r="M23" s="16">
+      <c r="L23" s="14">
+        <v>100</v>
+      </c>
+      <c r="M23" s="15">
         <v>7.2830000000000006E-2</v>
       </c>
-      <c r="N23" s="16">
+      <c r="N23" s="15">
         <v>6.3530000000000003E-2</v>
       </c>
-      <c r="O23" s="17">
+      <c r="O23" s="16">
         <v>67.37</v>
       </c>
-      <c r="P23" s="15">
-        <v>100</v>
-      </c>
-      <c r="Q23" s="16">
+      <c r="P23" s="14">
+        <v>100</v>
+      </c>
+      <c r="Q23" s="15">
         <v>9.9860000000000004E-2</v>
       </c>
-      <c r="R23" s="16">
+      <c r="R23" s="15">
         <v>0.11802</v>
       </c>
-      <c r="S23" s="17">
+      <c r="S23" s="16">
         <v>66.290000000000006</v>
       </c>
     </row>
     <row r="24" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B24" s="18">
+      <c r="B24" s="17">
         <v>4</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24" s="31">
         <v>2454</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="8">
         <v>63</v>
       </c>
-      <c r="E24" s="10">
+      <c r="E24" s="9">
         <v>0.36531000000000002</v>
       </c>
-      <c r="F24" s="10">
+      <c r="F24" s="9">
         <v>1.58148</v>
       </c>
-      <c r="G24" s="11">
+      <c r="G24" s="10">
         <v>110.65</v>
       </c>
-      <c r="H24" s="9">
-        <v>100</v>
-      </c>
-      <c r="I24" s="10">
+      <c r="H24" s="8">
+        <v>100</v>
+      </c>
+      <c r="I24" s="9">
         <v>0.59524999999999995</v>
       </c>
-      <c r="J24" s="10">
+      <c r="J24" s="9">
         <v>1.19604</v>
       </c>
-      <c r="K24" s="11">
+      <c r="K24" s="10">
         <v>139.82</v>
       </c>
-      <c r="L24" s="9">
-        <v>100</v>
-      </c>
-      <c r="M24" s="10">
+      <c r="L24" s="8">
+        <v>100</v>
+      </c>
+      <c r="M24" s="9">
         <v>2.7779999999999999E-2</v>
       </c>
-      <c r="N24" s="10">
+      <c r="N24" s="9">
         <v>0.13266</v>
       </c>
-      <c r="O24" s="11">
+      <c r="O24" s="10">
         <v>5.46</v>
       </c>
-      <c r="P24" s="10">
-        <v>100</v>
-      </c>
-      <c r="Q24" s="10">
+      <c r="P24" s="9">
+        <v>100</v>
+      </c>
+      <c r="Q24" s="9">
         <v>7.7369999999999994E-2</v>
       </c>
-      <c r="R24" s="10">
+      <c r="R24" s="9">
         <v>0.35729</v>
       </c>
-      <c r="S24" s="11">
+      <c r="S24" s="10">
         <v>9.86</v>
       </c>
     </row>
     <row r="25" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B25" s="19">
+      <c r="B25" s="18">
         <v>4</v>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="32">
         <v>2390</v>
       </c>
-      <c r="D25" s="12">
+      <c r="D25" s="11">
         <v>67</v>
       </c>
       <c r="E25">
@@ -2099,10 +2138,10 @@
       <c r="F25">
         <v>5.1490200000000002</v>
       </c>
-      <c r="G25" s="14">
+      <c r="G25" s="13">
         <v>722.99</v>
       </c>
-      <c r="H25" s="12">
+      <c r="H25" s="11">
         <v>97</v>
       </c>
       <c r="I25">
@@ -2111,10 +2150,10 @@
       <c r="J25">
         <v>5.4575100000000001</v>
       </c>
-      <c r="K25" s="14">
+      <c r="K25" s="13">
         <v>1068.69</v>
       </c>
-      <c r="L25" s="12">
+      <c r="L25" s="11">
         <v>91</v>
       </c>
       <c r="M25">
@@ -2123,7 +2162,7 @@
       <c r="N25">
         <v>2.9720200000000001</v>
       </c>
-      <c r="O25" s="14">
+      <c r="O25" s="13">
         <v>138.6</v>
       </c>
       <c r="P25">
@@ -2135,18 +2174,18 @@
       <c r="R25">
         <v>3.0889799999999998</v>
       </c>
-      <c r="S25" s="14">
+      <c r="S25" s="13">
         <v>118.09</v>
       </c>
     </row>
     <row r="26" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="19">
+      <c r="B26" s="18">
         <v>4</v>
       </c>
-      <c r="C26" s="20">
+      <c r="C26" s="32">
         <v>2357</v>
       </c>
-      <c r="D26" s="12">
+      <c r="D26" s="11">
         <v>70</v>
       </c>
       <c r="E26">
@@ -2155,10 +2194,10 @@
       <c r="F26">
         <v>2.9649299999999998</v>
       </c>
-      <c r="G26" s="14">
+      <c r="G26" s="13">
         <v>237.74</v>
       </c>
-      <c r="H26" s="12">
+      <c r="H26" s="11">
         <v>99</v>
       </c>
       <c r="I26">
@@ -2167,10 +2206,10 @@
       <c r="J26">
         <v>3.3431600000000001</v>
       </c>
-      <c r="K26" s="14">
+      <c r="K26" s="13">
         <v>383.9</v>
       </c>
-      <c r="L26" s="12">
+      <c r="L26" s="11">
         <v>100</v>
       </c>
       <c r="M26">
@@ -2179,7 +2218,7 @@
       <c r="N26">
         <v>0.44885000000000003</v>
       </c>
-      <c r="O26" s="14">
+      <c r="O26" s="13">
         <v>27.08</v>
       </c>
       <c r="P26">
@@ -2191,18 +2230,18 @@
       <c r="R26">
         <v>0.60663</v>
       </c>
-      <c r="S26" s="14">
+      <c r="S26" s="13">
         <v>27.98</v>
       </c>
     </row>
     <row r="27" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B27" s="19">
+      <c r="B27" s="18">
         <v>4</v>
       </c>
-      <c r="C27" s="20">
+      <c r="C27" s="32">
         <v>2350</v>
       </c>
-      <c r="D27" s="12">
+      <c r="D27" s="11">
         <v>77</v>
       </c>
       <c r="E27">
@@ -2211,10 +2250,10 @@
       <c r="F27">
         <v>2.0596999999999999</v>
       </c>
-      <c r="G27" s="14">
+      <c r="G27" s="13">
         <v>142.22999999999999</v>
       </c>
-      <c r="H27" s="12">
+      <c r="H27" s="11">
         <v>100</v>
       </c>
       <c r="I27">
@@ -2223,10 +2262,10 @@
       <c r="J27">
         <v>0.93906000000000001</v>
       </c>
-      <c r="K27" s="14">
+      <c r="K27" s="13">
         <v>152.80000000000001</v>
       </c>
-      <c r="L27" s="12">
+      <c r="L27" s="11">
         <v>100</v>
       </c>
       <c r="M27">
@@ -2235,7 +2274,7 @@
       <c r="N27">
         <v>0.14252999999999999</v>
       </c>
-      <c r="O27" s="14">
+      <c r="O27" s="13">
         <v>7.73</v>
       </c>
       <c r="P27">
@@ -2247,18 +2286,18 @@
       <c r="R27">
         <v>4.2199999999999998E-3</v>
       </c>
-      <c r="S27" s="14">
+      <c r="S27" s="13">
         <v>3.38</v>
       </c>
     </row>
     <row r="28" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B28" s="19">
+      <c r="B28" s="18">
         <v>4</v>
       </c>
-      <c r="C28" s="20">
+      <c r="C28" s="32">
         <v>2563</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="11">
         <v>78</v>
       </c>
       <c r="E28">
@@ -2267,10 +2306,10 @@
       <c r="F28">
         <v>0.39439000000000002</v>
       </c>
-      <c r="G28" s="14">
+      <c r="G28" s="13">
         <v>38.630000000000003</v>
       </c>
-      <c r="H28" s="12">
+      <c r="H28" s="11">
         <v>100</v>
       </c>
       <c r="I28">
@@ -2279,10 +2318,10 @@
       <c r="J28">
         <v>0.38108999999999998</v>
       </c>
-      <c r="K28" s="14">
+      <c r="K28" s="13">
         <v>41.77</v>
       </c>
-      <c r="L28" s="12">
+      <c r="L28" s="11">
         <v>100</v>
       </c>
       <c r="M28">
@@ -2291,7 +2330,7 @@
       <c r="N28">
         <v>1.2869999999999999E-2</v>
       </c>
-      <c r="O28" s="14">
+      <c r="O28" s="13">
         <v>4</v>
       </c>
       <c r="P28">
@@ -2303,18 +2342,18 @@
       <c r="R28">
         <v>1.018E-2</v>
       </c>
-      <c r="S28" s="14">
+      <c r="S28" s="13">
         <v>4.04</v>
       </c>
     </row>
     <row r="29" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B29" s="19">
+      <c r="B29" s="18">
         <v>4</v>
       </c>
-      <c r="C29" s="20">
+      <c r="C29" s="32">
         <v>2456</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="11">
         <v>81</v>
       </c>
       <c r="E29">
@@ -2323,10 +2362,10 @@
       <c r="F29">
         <v>0.44784000000000002</v>
       </c>
-      <c r="G29" s="14">
+      <c r="G29" s="13">
         <v>38.17</v>
       </c>
-      <c r="H29" s="12">
+      <c r="H29" s="11">
         <v>100</v>
       </c>
       <c r="I29">
@@ -2335,10 +2374,10 @@
       <c r="J29">
         <v>1.6574199999999999</v>
       </c>
-      <c r="K29" s="14">
+      <c r="K29" s="13">
         <v>67.290000000000006</v>
       </c>
-      <c r="L29" s="12">
+      <c r="L29" s="11">
         <v>100</v>
       </c>
       <c r="M29">
@@ -2347,7 +2386,7 @@
       <c r="N29">
         <v>2.0830000000000001E-2</v>
       </c>
-      <c r="O29" s="14">
+      <c r="O29" s="13">
         <v>2.96</v>
       </c>
       <c r="P29">
@@ -2359,18 +2398,18 @@
       <c r="R29">
         <v>8.2890000000000005E-2</v>
       </c>
-      <c r="S29" s="14">
+      <c r="S29" s="13">
         <v>3.76</v>
       </c>
     </row>
     <row r="30" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B30" s="19">
+      <c r="B30" s="18">
         <v>4</v>
       </c>
-      <c r="C30" s="20">
+      <c r="C30" s="32">
         <v>2525</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="11">
         <v>83</v>
       </c>
       <c r="E30">
@@ -2379,10 +2418,10 @@
       <c r="F30">
         <v>2.82491</v>
       </c>
-      <c r="G30" s="14">
+      <c r="G30" s="13">
         <v>579.99</v>
       </c>
-      <c r="H30" s="12">
+      <c r="H30" s="11">
         <v>100</v>
       </c>
       <c r="I30">
@@ -2391,10 +2430,10 @@
       <c r="J30">
         <v>3.2895599999999998</v>
       </c>
-      <c r="K30" s="14">
+      <c r="K30" s="13">
         <v>477.73</v>
       </c>
-      <c r="L30" s="12">
+      <c r="L30" s="11">
         <v>100</v>
       </c>
       <c r="M30">
@@ -2403,7 +2442,7 @@
       <c r="N30">
         <v>0.24954000000000001</v>
       </c>
-      <c r="O30" s="14">
+      <c r="O30" s="13">
         <v>23.16</v>
       </c>
       <c r="P30">
@@ -2415,18 +2454,18 @@
       <c r="R30">
         <v>0.36280000000000001</v>
       </c>
-      <c r="S30" s="14">
+      <c r="S30" s="13">
         <v>22.24</v>
       </c>
     </row>
     <row r="31" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B31" s="19">
+      <c r="B31" s="18">
         <v>4</v>
       </c>
-      <c r="C31" s="20">
+      <c r="C31" s="32">
         <v>2405</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="11">
         <v>86</v>
       </c>
       <c r="E31">
@@ -2435,10 +2474,10 @@
       <c r="F31">
         <v>3.4679500000000001</v>
       </c>
-      <c r="G31" s="14">
+      <c r="G31" s="13">
         <v>813.59</v>
       </c>
-      <c r="H31" s="12">
+      <c r="H31" s="11">
         <v>100</v>
       </c>
       <c r="I31">
@@ -2447,10 +2486,10 @@
       <c r="J31">
         <v>3.9477899999999999</v>
       </c>
-      <c r="K31" s="14">
+      <c r="K31" s="13">
         <v>808.31</v>
       </c>
-      <c r="L31" s="12">
+      <c r="L31" s="11">
         <v>100</v>
       </c>
       <c r="M31">
@@ -2459,7 +2498,7 @@
       <c r="N31">
         <v>1.431</v>
       </c>
-      <c r="O31" s="14">
+      <c r="O31" s="13">
         <v>164.62</v>
       </c>
       <c r="P31">
@@ -2471,18 +2510,18 @@
       <c r="R31">
         <v>2.1948699999999999</v>
       </c>
-      <c r="S31" s="14">
+      <c r="S31" s="13">
         <v>130.13999999999999</v>
       </c>
     </row>
     <row r="32" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="19">
+      <c r="B32" s="18">
         <v>4</v>
       </c>
-      <c r="C32" s="20">
+      <c r="C32" s="32">
         <v>2281</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="11">
         <v>88</v>
       </c>
       <c r="E32">
@@ -2491,10 +2530,10 @@
       <c r="F32">
         <v>0.50438000000000005</v>
       </c>
-      <c r="G32" s="14">
+      <c r="G32" s="13">
         <v>51.97</v>
       </c>
-      <c r="H32" s="12">
+      <c r="H32" s="11">
         <v>100</v>
       </c>
       <c r="I32">
@@ -2503,10 +2542,10 @@
       <c r="J32">
         <v>0.49169000000000002</v>
       </c>
-      <c r="K32" s="14">
+      <c r="K32" s="13">
         <v>58.01</v>
       </c>
-      <c r="L32" s="12">
+      <c r="L32" s="11">
         <v>100</v>
       </c>
       <c r="M32">
@@ -2515,7 +2554,7 @@
       <c r="N32">
         <v>6.8599999999999998E-3</v>
       </c>
-      <c r="O32" s="14">
+      <c r="O32" s="13">
         <v>3.82</v>
       </c>
       <c r="P32">
@@ -2527,18 +2566,18 @@
       <c r="R32">
         <v>9.7999999999999997E-3</v>
       </c>
-      <c r="S32" s="14">
+      <c r="S32" s="13">
         <v>3.56</v>
       </c>
     </row>
     <row r="33" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B33" s="19">
+      <c r="B33" s="18">
         <v>4</v>
       </c>
-      <c r="C33" s="20">
+      <c r="C33" s="32">
         <v>2862</v>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="11">
         <v>88</v>
       </c>
       <c r="E33">
@@ -2547,10 +2586,10 @@
       <c r="F33">
         <v>4.7191400000000003</v>
       </c>
-      <c r="G33" s="14">
+      <c r="G33" s="13">
         <v>1007.3</v>
       </c>
-      <c r="H33" s="12">
+      <c r="H33" s="11">
         <v>99</v>
       </c>
       <c r="I33">
@@ -2559,10 +2598,10 @@
       <c r="J33">
         <v>2.9992200000000002</v>
       </c>
-      <c r="K33" s="14">
+      <c r="K33" s="13">
         <v>399.49</v>
       </c>
-      <c r="L33" s="12">
+      <c r="L33" s="11">
         <v>100</v>
       </c>
       <c r="M33">
@@ -2571,7 +2610,7 @@
       <c r="N33">
         <v>0.89009000000000005</v>
       </c>
-      <c r="O33" s="14">
+      <c r="O33" s="13">
         <v>23.53</v>
       </c>
       <c r="P33">
@@ -2583,18 +2622,18 @@
       <c r="R33">
         <v>0.45468999999999998</v>
       </c>
-      <c r="S33" s="14">
+      <c r="S33" s="13">
         <v>19.38</v>
       </c>
     </row>
     <row r="34" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B34" s="19">
+      <c r="B34" s="18">
         <v>4</v>
       </c>
-      <c r="C34" s="20">
+      <c r="C34" s="19">
         <v>2755</v>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="11">
         <v>89</v>
       </c>
       <c r="E34">
@@ -2603,10 +2642,10 @@
       <c r="F34">
         <v>3.7179799999999998</v>
       </c>
-      <c r="G34" s="14">
+      <c r="G34" s="13">
         <v>876.21</v>
       </c>
-      <c r="H34" s="12">
+      <c r="H34" s="11">
         <v>100</v>
       </c>
       <c r="I34">
@@ -2615,10 +2654,10 @@
       <c r="J34">
         <v>2.60487</v>
       </c>
-      <c r="K34" s="14">
+      <c r="K34" s="13">
         <v>356.39</v>
       </c>
-      <c r="L34" s="12">
+      <c r="L34" s="11">
         <v>100</v>
       </c>
       <c r="M34">
@@ -2627,7 +2666,7 @@
       <c r="N34">
         <v>0.38533000000000001</v>
       </c>
-      <c r="O34" s="14">
+      <c r="O34" s="13">
         <v>24.82</v>
       </c>
       <c r="P34">
@@ -2639,18 +2678,18 @@
       <c r="R34">
         <v>0.37203000000000003</v>
       </c>
-      <c r="S34" s="14">
+      <c r="S34" s="13">
         <v>24.85</v>
       </c>
     </row>
     <row r="35" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B35" s="19">
+      <c r="B35" s="18">
         <v>4</v>
       </c>
-      <c r="C35" s="20">
+      <c r="C35" s="19">
         <v>2349</v>
       </c>
-      <c r="D35" s="12">
+      <c r="D35" s="11">
         <v>90</v>
       </c>
       <c r="E35">
@@ -2659,10 +2698,10 @@
       <c r="F35">
         <v>4.1051799999999998</v>
       </c>
-      <c r="G35" s="14">
+      <c r="G35" s="13">
         <v>484.07</v>
       </c>
-      <c r="H35" s="12">
+      <c r="H35" s="11">
         <v>100</v>
       </c>
       <c r="I35">
@@ -2671,10 +2710,10 @@
       <c r="J35">
         <v>2.1403300000000001</v>
       </c>
-      <c r="K35" s="14">
+      <c r="K35" s="13">
         <v>366.52</v>
       </c>
-      <c r="L35" s="12">
+      <c r="L35" s="11">
         <v>100</v>
       </c>
       <c r="M35">
@@ -2683,7 +2722,7 @@
       <c r="N35">
         <v>0.41276000000000002</v>
       </c>
-      <c r="O35" s="14">
+      <c r="O35" s="13">
         <v>56.72</v>
       </c>
       <c r="P35">
@@ -2695,18 +2734,18 @@
       <c r="R35">
         <v>1.54051</v>
       </c>
-      <c r="S35" s="14">
+      <c r="S35" s="13">
         <v>53.11</v>
       </c>
     </row>
     <row r="36" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B36" s="19">
+      <c r="B36" s="18">
         <v>4</v>
       </c>
-      <c r="C36" s="20">
+      <c r="C36" s="19">
         <v>2851</v>
       </c>
-      <c r="D36" s="12">
+      <c r="D36" s="11">
         <v>90</v>
       </c>
       <c r="E36">
@@ -2715,10 +2754,10 @@
       <c r="F36">
         <v>3.1205400000000001</v>
       </c>
-      <c r="G36" s="14">
+      <c r="G36" s="13">
         <v>580.26</v>
       </c>
-      <c r="H36" s="12">
+      <c r="H36" s="11">
         <v>100</v>
       </c>
       <c r="I36">
@@ -2727,10 +2766,10 @@
       <c r="J36">
         <v>2.0628299999999999</v>
       </c>
-      <c r="K36" s="14">
+      <c r="K36" s="13">
         <v>355.66</v>
       </c>
-      <c r="L36" s="12">
+      <c r="L36" s="11">
         <v>100</v>
       </c>
       <c r="M36">
@@ -2739,7 +2778,7 @@
       <c r="N36">
         <v>0.28683999999999998</v>
       </c>
-      <c r="O36" s="14">
+      <c r="O36" s="13">
         <v>32.770000000000003</v>
       </c>
       <c r="P36">
@@ -2751,18 +2790,18 @@
       <c r="R36">
         <v>0.33173999999999998</v>
       </c>
-      <c r="S36" s="14">
+      <c r="S36" s="13">
         <v>33.35</v>
       </c>
     </row>
     <row r="37" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B37" s="19">
+      <c r="B37" s="18">
         <v>4</v>
       </c>
-      <c r="C37" s="20">
+      <c r="C37" s="19">
         <v>2233</v>
       </c>
-      <c r="D37" s="12">
+      <c r="D37" s="11">
         <v>91</v>
       </c>
       <c r="E37">
@@ -2771,10 +2810,10 @@
       <c r="F37">
         <v>1.57178</v>
       </c>
-      <c r="G37" s="14">
+      <c r="G37" s="13">
         <v>138.99</v>
       </c>
-      <c r="H37" s="12">
+      <c r="H37" s="11">
         <v>100</v>
       </c>
       <c r="I37">
@@ -2783,10 +2822,10 @@
       <c r="J37">
         <v>2.16384</v>
       </c>
-      <c r="K37" s="14">
+      <c r="K37" s="13">
         <v>261.32</v>
       </c>
-      <c r="L37" s="12">
+      <c r="L37" s="11">
         <v>100</v>
       </c>
       <c r="M37">
@@ -2795,7 +2834,7 @@
       <c r="N37">
         <v>1.6279999999999999E-2</v>
       </c>
-      <c r="O37" s="14">
+      <c r="O37" s="13">
         <v>4.5599999999999996</v>
       </c>
       <c r="P37">
@@ -2807,18 +2846,18 @@
       <c r="R37">
         <v>7.5620000000000007E-2</v>
       </c>
-      <c r="S37" s="14">
+      <c r="S37" s="13">
         <v>6.84</v>
       </c>
     </row>
     <row r="38" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B38" s="19">
+      <c r="B38" s="18">
         <v>4</v>
       </c>
-      <c r="C38" s="20">
+      <c r="C38" s="19">
         <v>2354</v>
       </c>
-      <c r="D38" s="12">
+      <c r="D38" s="11">
         <v>91</v>
       </c>
       <c r="E38">
@@ -2827,10 +2866,10 @@
       <c r="F38">
         <v>3.6515399999999998</v>
       </c>
-      <c r="G38" s="14">
+      <c r="G38" s="13">
         <v>845.93</v>
       </c>
-      <c r="H38" s="12">
+      <c r="H38" s="11">
         <v>100</v>
       </c>
       <c r="I38">
@@ -2839,10 +2878,10 @@
       <c r="J38">
         <v>2.4450799999999999</v>
       </c>
-      <c r="K38" s="14">
+      <c r="K38" s="13">
         <v>471.65</v>
       </c>
-      <c r="L38" s="12">
+      <c r="L38" s="11">
         <v>100</v>
       </c>
       <c r="M38">
@@ -2851,7 +2890,7 @@
       <c r="N38">
         <v>2.05627</v>
       </c>
-      <c r="O38" s="14">
+      <c r="O38" s="13">
         <v>220.2</v>
       </c>
       <c r="P38">
@@ -2863,18 +2902,18 @@
       <c r="R38">
         <v>2.3488000000000002</v>
       </c>
-      <c r="S38" s="14">
+      <c r="S38" s="13">
         <v>151.22</v>
       </c>
     </row>
     <row r="39" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B39" s="19">
+      <c r="B39" s="18">
         <v>4</v>
       </c>
-      <c r="C39" s="20">
+      <c r="C39" s="19">
         <v>2571</v>
       </c>
-      <c r="D39" s="12">
+      <c r="D39" s="11">
         <v>91</v>
       </c>
       <c r="E39">
@@ -2883,10 +2922,10 @@
       <c r="F39">
         <v>5.0979999999999998E-2</v>
       </c>
-      <c r="G39" s="14">
+      <c r="G39" s="13">
         <v>12.71</v>
       </c>
-      <c r="H39" s="12">
+      <c r="H39" s="11">
         <v>100</v>
       </c>
       <c r="I39">
@@ -2895,10 +2934,10 @@
       <c r="J39">
         <v>0.94123999999999997</v>
       </c>
-      <c r="K39" s="14">
+      <c r="K39" s="13">
         <v>68.3</v>
       </c>
-      <c r="L39" s="12">
+      <c r="L39" s="11">
         <v>100</v>
       </c>
       <c r="M39">
@@ -2907,7 +2946,7 @@
       <c r="N39">
         <v>8.8999999999999999E-3</v>
       </c>
-      <c r="O39" s="14">
+      <c r="O39" s="13">
         <v>3.44</v>
       </c>
       <c r="P39">
@@ -2919,18 +2958,18 @@
       <c r="R39">
         <v>1.523E-2</v>
       </c>
-      <c r="S39" s="14">
+      <c r="S39" s="13">
         <v>3.55</v>
       </c>
     </row>
     <row r="40" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B40" s="19">
+      <c r="B40" s="18">
         <v>4</v>
       </c>
-      <c r="C40" s="20">
+      <c r="C40" s="19">
         <v>2602</v>
       </c>
-      <c r="D40" s="12">
+      <c r="D40" s="11">
         <v>91</v>
       </c>
       <c r="E40">
@@ -2939,10 +2978,10 @@
       <c r="F40">
         <v>2.76702</v>
       </c>
-      <c r="G40" s="14">
+      <c r="G40" s="13">
         <v>383.32</v>
       </c>
-      <c r="H40" s="12">
+      <c r="H40" s="11">
         <v>100</v>
       </c>
       <c r="I40">
@@ -2951,10 +2990,10 @@
       <c r="J40">
         <v>1.5324899999999999</v>
       </c>
-      <c r="K40" s="14">
+      <c r="K40" s="13">
         <v>197.78</v>
       </c>
-      <c r="L40" s="12">
+      <c r="L40" s="11">
         <v>100</v>
       </c>
       <c r="M40">
@@ -2963,7 +3002,7 @@
       <c r="N40">
         <v>0.35531000000000001</v>
       </c>
-      <c r="O40" s="14">
+      <c r="O40" s="13">
         <v>41.18</v>
       </c>
       <c r="P40">
@@ -2975,18 +3014,18 @@
       <c r="R40">
         <v>0.3841</v>
       </c>
-      <c r="S40" s="14">
+      <c r="S40" s="13">
         <v>31.81</v>
       </c>
     </row>
     <row r="41" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B41" s="19">
+      <c r="B41" s="18">
         <v>4</v>
       </c>
-      <c r="C41" s="20">
+      <c r="C41" s="19">
         <v>2467</v>
       </c>
-      <c r="D41" s="12">
+      <c r="D41" s="11">
         <v>92</v>
       </c>
       <c r="E41">
@@ -2995,10 +3034,10 @@
       <c r="F41">
         <v>1.9658100000000001</v>
       </c>
-      <c r="G41" s="14">
+      <c r="G41" s="13">
         <v>270.93</v>
       </c>
-      <c r="H41" s="12">
+      <c r="H41" s="11">
         <v>100</v>
       </c>
       <c r="I41">
@@ -3007,10 +3046,10 @@
       <c r="J41">
         <v>0.61960999999999999</v>
       </c>
-      <c r="K41" s="14">
+      <c r="K41" s="13">
         <v>65.05</v>
       </c>
-      <c r="L41" s="12">
+      <c r="L41" s="11">
         <v>100</v>
       </c>
       <c r="M41">
@@ -3019,7 +3058,7 @@
       <c r="N41">
         <v>1.2019999999999999E-2</v>
       </c>
-      <c r="O41" s="14">
+      <c r="O41" s="13">
         <v>3.46</v>
       </c>
       <c r="P41">
@@ -3031,18 +3070,18 @@
       <c r="R41">
         <v>1.1560000000000001E-2</v>
       </c>
-      <c r="S41" s="14">
+      <c r="S41" s="13">
         <v>3.74</v>
       </c>
     </row>
     <row r="42" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B42" s="19">
+      <c r="B42" s="18">
         <v>4</v>
       </c>
-      <c r="C42" s="20">
+      <c r="C42" s="19">
         <v>2985</v>
       </c>
-      <c r="D42" s="12">
+      <c r="D42" s="11">
         <v>92</v>
       </c>
       <c r="E42">
@@ -3051,10 +3090,10 @@
       <c r="F42">
         <v>2.85425</v>
       </c>
-      <c r="G42" s="14">
+      <c r="G42" s="13">
         <v>355.36</v>
       </c>
-      <c r="H42" s="12">
+      <c r="H42" s="11">
         <v>100</v>
       </c>
       <c r="I42">
@@ -3063,10 +3102,10 @@
       <c r="J42">
         <v>1.2023200000000001</v>
       </c>
-      <c r="K42" s="14">
+      <c r="K42" s="13">
         <v>126.7</v>
       </c>
-      <c r="L42" s="12">
+      <c r="L42" s="11">
         <v>100</v>
       </c>
       <c r="M42">
@@ -3075,7 +3114,7 @@
       <c r="N42">
         <v>0.30164000000000002</v>
       </c>
-      <c r="O42" s="14">
+      <c r="O42" s="13">
         <v>12.89</v>
       </c>
       <c r="P42">
@@ -3087,130 +3126,130 @@
       <c r="R42">
         <v>0.10105</v>
       </c>
-      <c r="S42" s="14">
+      <c r="S42" s="13">
         <v>9.1</v>
       </c>
     </row>
     <row r="43" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B43" s="21">
+      <c r="B43" s="20">
         <v>4</v>
       </c>
-      <c r="C43" s="4">
+      <c r="C43" s="3">
         <v>2292</v>
       </c>
-      <c r="D43" s="15">
+      <c r="D43" s="14">
         <v>93</v>
       </c>
-      <c r="E43" s="16">
+      <c r="E43" s="15">
         <v>20.268270000000001</v>
       </c>
-      <c r="F43" s="16">
+      <c r="F43" s="15">
         <v>188.26946000000001</v>
       </c>
-      <c r="G43" s="17">
+      <c r="G43" s="16">
         <v>115.54</v>
       </c>
-      <c r="H43" s="15">
-        <v>100</v>
-      </c>
-      <c r="I43" s="16">
+      <c r="H43" s="14">
+        <v>100</v>
+      </c>
+      <c r="I43" s="15">
         <v>0.38205</v>
       </c>
-      <c r="J43" s="16">
+      <c r="J43" s="15">
         <v>0.73004999999999998</v>
       </c>
-      <c r="K43" s="17">
+      <c r="K43" s="16">
         <v>105.05</v>
       </c>
-      <c r="L43" s="15">
-        <v>100</v>
-      </c>
-      <c r="M43" s="16">
+      <c r="L43" s="14">
+        <v>100</v>
+      </c>
+      <c r="M43" s="15">
         <v>2.256E-2</v>
       </c>
-      <c r="N43" s="16">
+      <c r="N43" s="15">
         <v>3.7260000000000001E-2</v>
       </c>
-      <c r="O43" s="17">
+      <c r="O43" s="16">
         <v>4.83</v>
       </c>
-      <c r="P43" s="16">
-        <v>100</v>
-      </c>
-      <c r="Q43" s="16">
+      <c r="P43" s="15">
+        <v>100</v>
+      </c>
+      <c r="Q43" s="15">
         <v>2.5669999999999998E-2</v>
       </c>
-      <c r="R43" s="16">
+      <c r="R43" s="15">
         <v>3.9969999999999999E-2</v>
       </c>
-      <c r="S43" s="17">
+      <c r="S43" s="16">
         <v>5.04</v>
       </c>
     </row>
     <row r="44" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B44" s="18">
+      <c r="B44" s="17">
         <v>5</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="D44" s="9">
+      <c r="D44" s="8">
         <v>22</v>
       </c>
-      <c r="E44" s="10">
+      <c r="E44" s="9">
         <v>3.4712000000000001</v>
       </c>
-      <c r="F44" s="10">
+      <c r="F44" s="9">
         <v>5.6835899999999997</v>
       </c>
-      <c r="G44" s="11">
+      <c r="G44" s="10">
         <v>140.86000000000001</v>
       </c>
-      <c r="H44" s="9">
+      <c r="H44" s="8">
         <v>36</v>
       </c>
-      <c r="I44" s="10">
+      <c r="I44" s="9">
         <v>22.113440000000001</v>
       </c>
-      <c r="J44" s="10">
+      <c r="J44" s="9">
         <v>26.34721</v>
       </c>
-      <c r="K44" s="11">
+      <c r="K44" s="10">
         <v>704.86</v>
       </c>
-      <c r="L44" s="9">
+      <c r="L44" s="8">
         <v>57</v>
       </c>
-      <c r="M44" s="10">
+      <c r="M44" s="9">
         <v>0.41363</v>
       </c>
-      <c r="N44" s="10">
+      <c r="N44" s="9">
         <v>0.97899999999999998</v>
       </c>
-      <c r="O44" s="11">
+      <c r="O44" s="10">
         <v>37.96</v>
       </c>
-      <c r="P44" s="10">
+      <c r="P44" s="9">
         <v>66</v>
       </c>
-      <c r="Q44" s="10">
+      <c r="Q44" s="9">
         <v>1.3809199999999999</v>
       </c>
-      <c r="R44" s="10">
+      <c r="R44" s="9">
         <v>4.98874</v>
       </c>
-      <c r="S44" s="11">
+      <c r="S44" s="10">
         <v>77.11</v>
       </c>
     </row>
     <row r="45" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B45" s="19">
+      <c r="B45" s="18">
         <v>5</v>
       </c>
-      <c r="C45" s="13" t="s">
+      <c r="C45" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="D45" s="12">
+      <c r="D45" s="11">
         <v>25</v>
       </c>
       <c r="E45">
@@ -3219,10 +3258,10 @@
       <c r="F45">
         <v>19.948340000000002</v>
       </c>
-      <c r="G45" s="14">
+      <c r="G45" s="13">
         <v>472.72</v>
       </c>
-      <c r="H45" s="12">
+      <c r="H45" s="11">
         <v>63</v>
       </c>
       <c r="I45">
@@ -3231,10 +3270,10 @@
       <c r="J45">
         <v>34.033540000000002</v>
       </c>
-      <c r="K45" s="14">
+      <c r="K45" s="13">
         <v>1144.71</v>
       </c>
-      <c r="L45" s="12">
+      <c r="L45" s="11">
         <v>71</v>
       </c>
       <c r="M45">
@@ -3243,7 +3282,7 @@
       <c r="N45">
         <v>21.96349</v>
       </c>
-      <c r="O45" s="14">
+      <c r="O45" s="13">
         <v>509.83</v>
       </c>
       <c r="P45">
@@ -3255,18 +3294,18 @@
       <c r="R45">
         <v>19.56982</v>
       </c>
-      <c r="S45" s="14">
+      <c r="S45" s="13">
         <v>474.3</v>
       </c>
     </row>
     <row r="46" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B46" s="19">
+      <c r="B46" s="18">
         <v>5</v>
       </c>
-      <c r="C46" s="13" t="s">
+      <c r="C46" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="D46" s="12">
+      <c r="D46" s="11">
         <v>28</v>
       </c>
       <c r="E46">
@@ -3275,10 +3314,10 @@
       <c r="F46">
         <v>33.390239999999999</v>
       </c>
-      <c r="G46" s="14">
+      <c r="G46" s="13">
         <v>907.25</v>
       </c>
-      <c r="H46" s="12">
+      <c r="H46" s="11">
         <v>33</v>
       </c>
       <c r="I46">
@@ -3287,10 +3326,10 @@
       <c r="J46">
         <v>31.964179999999999</v>
       </c>
-      <c r="K46" s="14">
+      <c r="K46" s="13">
         <v>1886.09</v>
       </c>
-      <c r="L46" s="12">
+      <c r="L46" s="11">
         <v>39</v>
       </c>
       <c r="M46">
@@ -3299,7 +3338,7 @@
       <c r="N46">
         <v>25.525510000000001</v>
       </c>
-      <c r="O46" s="14">
+      <c r="O46" s="13">
         <v>583.08000000000004</v>
       </c>
       <c r="P46">
@@ -3311,18 +3350,18 @@
       <c r="R46">
         <v>28.81851</v>
       </c>
-      <c r="S46" s="14">
+      <c r="S46" s="13">
         <v>704.2</v>
       </c>
     </row>
     <row r="47" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B47" s="19">
+      <c r="B47" s="18">
         <v>5</v>
       </c>
-      <c r="C47" s="13" t="s">
+      <c r="C47" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="D47" s="12">
+      <c r="D47" s="11">
         <v>34</v>
       </c>
       <c r="E47">
@@ -3331,10 +3370,10 @@
       <c r="F47">
         <v>33.40211</v>
       </c>
-      <c r="G47" s="14">
+      <c r="G47" s="13">
         <v>895.53</v>
       </c>
-      <c r="H47" s="12">
+      <c r="H47" s="11">
         <v>61</v>
       </c>
       <c r="I47">
@@ -3343,10 +3382,10 @@
       <c r="J47">
         <v>33.114870000000003</v>
       </c>
-      <c r="K47" s="14">
+      <c r="K47" s="13">
         <v>1189.93</v>
       </c>
-      <c r="L47" s="12">
+      <c r="L47" s="11">
         <v>74</v>
       </c>
       <c r="M47">
@@ -3355,7 +3394,7 @@
       <c r="N47">
         <v>14.474769999999999</v>
       </c>
-      <c r="O47" s="14">
+      <c r="O47" s="13">
         <v>340.97</v>
       </c>
       <c r="P47">
@@ -3367,18 +3406,18 @@
       <c r="R47">
         <v>24.54796</v>
       </c>
-      <c r="S47" s="14">
+      <c r="S47" s="13">
         <v>588.41</v>
       </c>
     </row>
     <row r="48" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B48" s="19">
+      <c r="B48" s="18">
         <v>5</v>
       </c>
-      <c r="C48" s="13" t="s">
+      <c r="C48" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="D48" s="12">
+      <c r="D48" s="11">
         <v>36</v>
       </c>
       <c r="E48">
@@ -3387,10 +3426,10 @@
       <c r="F48">
         <v>26.94426</v>
       </c>
-      <c r="G48" s="14">
+      <c r="G48" s="13">
         <v>662</v>
       </c>
-      <c r="H48" s="12">
+      <c r="H48" s="11">
         <v>82</v>
       </c>
       <c r="I48">
@@ -3399,10 +3438,10 @@
       <c r="J48">
         <v>32.17098</v>
       </c>
-      <c r="K48" s="14">
+      <c r="K48" s="13">
         <v>1023.8</v>
       </c>
-      <c r="L48" s="12">
+      <c r="L48" s="11">
         <v>76</v>
       </c>
       <c r="M48">
@@ -3411,7 +3450,7 @@
       <c r="N48">
         <v>23.412659999999999</v>
       </c>
-      <c r="O48" s="14">
+      <c r="O48" s="13">
         <v>533.58000000000004</v>
       </c>
       <c r="P48">
@@ -3423,18 +3462,18 @@
       <c r="R48">
         <v>13.470039999999999</v>
       </c>
-      <c r="S48" s="14">
+      <c r="S48" s="13">
         <v>321.14</v>
       </c>
     </row>
     <row r="49" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B49" s="19">
+      <c r="B49" s="18">
         <v>5</v>
       </c>
-      <c r="C49" s="13" t="s">
+      <c r="C49" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="D49" s="12">
+      <c r="D49" s="11">
         <v>40</v>
       </c>
       <c r="E49">
@@ -3443,10 +3482,10 @@
       <c r="F49">
         <v>28.03689</v>
       </c>
-      <c r="G49" s="14">
+      <c r="G49" s="13">
         <v>719.98</v>
       </c>
-      <c r="H49" s="12">
+      <c r="H49" s="11">
         <v>75</v>
       </c>
       <c r="I49">
@@ -3455,10 +3494,10 @@
       <c r="J49">
         <v>30.263500000000001</v>
       </c>
-      <c r="K49" s="14">
+      <c r="K49" s="13">
         <v>944.47</v>
       </c>
-      <c r="L49" s="12">
+      <c r="L49" s="11">
         <v>85</v>
       </c>
       <c r="M49">
@@ -3467,7 +3506,7 @@
       <c r="N49">
         <v>20.773440000000001</v>
       </c>
-      <c r="O49" s="14">
+      <c r="O49" s="13">
         <v>539.16</v>
       </c>
       <c r="P49">
@@ -3479,18 +3518,18 @@
       <c r="R49">
         <v>16.318069999999999</v>
       </c>
-      <c r="S49" s="14">
+      <c r="S49" s="13">
         <v>378.33</v>
       </c>
     </row>
     <row r="50" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B50" s="19">
+      <c r="B50" s="18">
         <v>5</v>
       </c>
-      <c r="C50" s="13" t="s">
+      <c r="C50" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="D50" s="12">
+      <c r="D50" s="11">
         <v>42</v>
       </c>
       <c r="E50">
@@ -3499,10 +3538,10 @@
       <c r="F50">
         <v>23.334389999999999</v>
       </c>
-      <c r="G50" s="14">
+      <c r="G50" s="13">
         <v>434.3</v>
       </c>
-      <c r="H50" s="12">
+      <c r="H50" s="11">
         <v>100</v>
       </c>
       <c r="I50">
@@ -3511,10 +3550,10 @@
       <c r="J50">
         <v>15.59056</v>
       </c>
-      <c r="K50" s="14">
+      <c r="K50" s="13">
         <v>270.04000000000002</v>
       </c>
-      <c r="L50" s="12">
+      <c r="L50" s="11">
         <v>100</v>
       </c>
       <c r="M50">
@@ -3523,7 +3562,7 @@
       <c r="N50">
         <v>1.12191</v>
       </c>
-      <c r="O50" s="14">
+      <c r="O50" s="13">
         <v>64.55</v>
       </c>
       <c r="P50">
@@ -3535,18 +3574,18 @@
       <c r="R50">
         <v>3.3472599999999999</v>
       </c>
-      <c r="S50" s="14">
+      <c r="S50" s="13">
         <v>81.56</v>
       </c>
     </row>
     <row r="51" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B51" s="19">
+      <c r="B51" s="18">
         <v>5</v>
       </c>
-      <c r="C51" s="13" t="s">
+      <c r="C51" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="D51" s="12">
+      <c r="D51" s="11">
         <v>42</v>
       </c>
       <c r="E51">
@@ -3555,10 +3594,10 @@
       <c r="F51">
         <v>24.385100000000001</v>
       </c>
-      <c r="G51" s="14">
+      <c r="G51" s="13">
         <v>315.48</v>
       </c>
-      <c r="H51" s="12">
+      <c r="H51" s="11">
         <v>71</v>
       </c>
       <c r="I51">
@@ -3567,10 +3606,10 @@
       <c r="J51">
         <v>28.887049999999999</v>
       </c>
-      <c r="K51" s="14">
+      <c r="K51" s="13">
         <v>531.41999999999996</v>
       </c>
-      <c r="L51" s="12">
+      <c r="L51" s="11">
         <v>84</v>
       </c>
       <c r="M51">
@@ -3579,7 +3618,7 @@
       <c r="N51">
         <v>15.83371</v>
       </c>
-      <c r="O51" s="14">
+      <c r="O51" s="13">
         <v>350.97</v>
       </c>
       <c r="P51">
@@ -3591,18 +3630,18 @@
       <c r="R51">
         <v>8.8228600000000004</v>
       </c>
-      <c r="S51" s="14">
+      <c r="S51" s="13">
         <v>65.55</v>
       </c>
     </row>
     <row r="52" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B52" s="19">
+      <c r="B52" s="18">
         <v>5</v>
       </c>
-      <c r="C52" s="13" t="s">
+      <c r="C52" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="D52" s="12">
+      <c r="D52" s="11">
         <v>43</v>
       </c>
       <c r="E52">
@@ -3611,10 +3650,10 @@
       <c r="F52">
         <v>27.913440000000001</v>
       </c>
-      <c r="G52" s="14">
+      <c r="G52" s="13">
         <v>892.6</v>
       </c>
-      <c r="H52" s="12">
+      <c r="H52" s="11">
         <v>72</v>
       </c>
       <c r="I52">
@@ -3623,10 +3662,10 @@
       <c r="J52">
         <v>34.467590000000001</v>
       </c>
-      <c r="K52" s="14">
+      <c r="K52" s="13">
         <v>1308.21</v>
       </c>
-      <c r="L52" s="12">
+      <c r="L52" s="11">
         <v>87</v>
       </c>
       <c r="M52">
@@ -3635,7 +3674,7 @@
       <c r="N52">
         <v>3.4722400000000002</v>
       </c>
-      <c r="O52" s="14">
+      <c r="O52" s="13">
         <v>141.79</v>
       </c>
       <c r="P52">
@@ -3647,18 +3686,18 @@
       <c r="R52">
         <v>11.25573</v>
       </c>
-      <c r="S52" s="14">
+      <c r="S52" s="13">
         <v>151.11000000000001</v>
       </c>
     </row>
     <row r="53" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B53" s="19">
+      <c r="B53" s="18">
         <v>5</v>
       </c>
-      <c r="C53" s="13" t="s">
+      <c r="C53" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="D53" s="12">
+      <c r="D53" s="11">
         <v>44</v>
       </c>
       <c r="E53">
@@ -3667,10 +3706,10 @@
       <c r="F53">
         <v>24.780169999999998</v>
       </c>
-      <c r="G53" s="14">
+      <c r="G53" s="13">
         <v>755.8</v>
       </c>
-      <c r="H53" s="12">
+      <c r="H53" s="11">
         <v>74</v>
       </c>
       <c r="I53">
@@ -3679,10 +3718,10 @@
       <c r="J53">
         <v>29.332419999999999</v>
       </c>
-      <c r="K53" s="14">
+      <c r="K53" s="13">
         <v>971.81</v>
       </c>
-      <c r="L53" s="12">
+      <c r="L53" s="11">
         <v>83</v>
       </c>
       <c r="M53">
@@ -3691,7 +3730,7 @@
       <c r="N53">
         <v>16.327680000000001</v>
       </c>
-      <c r="O53" s="14">
+      <c r="O53" s="13">
         <v>476.68</v>
       </c>
       <c r="P53">
@@ -3703,18 +3742,18 @@
       <c r="R53">
         <v>17.405080000000002</v>
       </c>
-      <c r="S53" s="14">
+      <c r="S53" s="13">
         <v>558.49</v>
       </c>
     </row>
     <row r="54" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B54" s="19">
+      <c r="B54" s="18">
         <v>5</v>
       </c>
-      <c r="C54" s="13" t="s">
+      <c r="C54" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="D54" s="12">
+      <c r="D54" s="11">
         <v>44</v>
       </c>
       <c r="E54">
@@ -3723,10 +3762,10 @@
       <c r="F54">
         <v>27.82114</v>
       </c>
-      <c r="G54" s="14">
+      <c r="G54" s="13">
         <v>844.89</v>
       </c>
-      <c r="H54" s="12">
+      <c r="H54" s="11">
         <v>75</v>
       </c>
       <c r="I54">
@@ -3735,10 +3774,10 @@
       <c r="J54">
         <v>32.933970000000002</v>
       </c>
-      <c r="K54" s="14">
+      <c r="K54" s="13">
         <v>1042.6400000000001</v>
       </c>
-      <c r="L54" s="12">
+      <c r="L54" s="11">
         <v>83</v>
       </c>
       <c r="M54">
@@ -3747,7 +3786,7 @@
       <c r="N54">
         <v>13.3033</v>
       </c>
-      <c r="O54" s="14">
+      <c r="O54" s="13">
         <v>265.56</v>
       </c>
       <c r="P54">
@@ -3759,18 +3798,18 @@
       <c r="R54">
         <v>18.497399999999999</v>
       </c>
-      <c r="S54" s="14">
+      <c r="S54" s="13">
         <v>437.12</v>
       </c>
     </row>
     <row r="55" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B55" s="19">
+      <c r="B55" s="18">
         <v>5</v>
       </c>
-      <c r="C55" s="13" t="s">
+      <c r="C55" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="D55" s="12">
+      <c r="D55" s="11">
         <v>45</v>
       </c>
       <c r="E55">
@@ -3779,10 +3818,10 @@
       <c r="F55">
         <v>20.9558</v>
       </c>
-      <c r="G55" s="14">
+      <c r="G55" s="13">
         <v>539.30999999999995</v>
       </c>
-      <c r="H55" s="12">
+      <c r="H55" s="11">
         <v>48</v>
       </c>
       <c r="I55">
@@ -3791,10 +3830,10 @@
       <c r="J55">
         <v>22.733000000000001</v>
       </c>
-      <c r="K55" s="14">
+      <c r="K55" s="13">
         <v>472.85</v>
       </c>
-      <c r="L55" s="12">
+      <c r="L55" s="11">
         <v>90</v>
       </c>
       <c r="M55">
@@ -3803,7 +3842,7 @@
       <c r="N55">
         <v>4.2445599999999999</v>
       </c>
-      <c r="O55" s="14">
+      <c r="O55" s="13">
         <v>122.74</v>
       </c>
       <c r="P55">
@@ -3815,18 +3854,18 @@
       <c r="R55">
         <v>5.0933900000000003</v>
       </c>
-      <c r="S55" s="14">
+      <c r="S55" s="13">
         <v>102.83</v>
       </c>
     </row>
     <row r="56" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B56" s="19">
+      <c r="B56" s="18">
         <v>5</v>
       </c>
-      <c r="C56" s="13" t="s">
+      <c r="C56" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="D56" s="12">
+      <c r="D56" s="11">
         <v>46</v>
       </c>
       <c r="E56">
@@ -3835,10 +3874,10 @@
       <c r="F56">
         <v>24.69538</v>
       </c>
-      <c r="G56" s="14">
+      <c r="G56" s="13">
         <v>526.89</v>
       </c>
-      <c r="H56" s="12">
+      <c r="H56" s="11">
         <v>84</v>
       </c>
       <c r="I56">
@@ -3847,10 +3886,10 @@
       <c r="J56">
         <v>32.329619999999998</v>
       </c>
-      <c r="K56" s="14">
+      <c r="K56" s="13">
         <v>869.5</v>
       </c>
-      <c r="L56" s="12">
+      <c r="L56" s="11">
         <v>85</v>
       </c>
       <c r="M56">
@@ -3859,7 +3898,7 @@
       <c r="N56">
         <v>18.360440000000001</v>
       </c>
-      <c r="O56" s="14">
+      <c r="O56" s="13">
         <v>463.81</v>
       </c>
       <c r="P56">
@@ -3871,18 +3910,18 @@
       <c r="R56">
         <v>21.32</v>
       </c>
-      <c r="S56" s="14">
+      <c r="S56" s="13">
         <v>489.4</v>
       </c>
     </row>
     <row r="57" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B57" s="19">
+      <c r="B57" s="18">
         <v>5</v>
       </c>
-      <c r="C57" s="13" t="s">
+      <c r="C57" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="D57" s="12">
+      <c r="D57" s="11">
         <v>46</v>
       </c>
       <c r="E57">
@@ -3891,10 +3930,10 @@
       <c r="F57">
         <v>26.13458</v>
       </c>
-      <c r="G57" s="14">
+      <c r="G57" s="13">
         <v>591.83000000000004</v>
       </c>
-      <c r="H57" s="12">
+      <c r="H57" s="11">
         <v>72</v>
       </c>
       <c r="I57">
@@ -3903,10 +3942,10 @@
       <c r="J57">
         <v>35.03875</v>
       </c>
-      <c r="K57" s="14">
+      <c r="K57" s="13">
         <v>1025.22</v>
       </c>
-      <c r="L57" s="12">
+      <c r="L57" s="11">
         <v>87</v>
       </c>
       <c r="M57">
@@ -3915,7 +3954,7 @@
       <c r="N57">
         <v>21.39537</v>
       </c>
-      <c r="O57" s="14">
+      <c r="O57" s="13">
         <v>429.13</v>
       </c>
       <c r="P57">
@@ -3927,18 +3966,18 @@
       <c r="R57">
         <v>9.5222999999999995</v>
       </c>
-      <c r="S57" s="14">
+      <c r="S57" s="13">
         <v>256.14999999999998</v>
       </c>
     </row>
     <row r="58" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="19">
+      <c r="B58" s="18">
         <v>5</v>
       </c>
-      <c r="C58" s="13" t="s">
+      <c r="C58" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="D58" s="12">
+      <c r="D58" s="11">
         <v>48</v>
       </c>
       <c r="E58">
@@ -3947,10 +3986,10 @@
       <c r="F58">
         <v>17.922640000000001</v>
       </c>
-      <c r="G58" s="14">
+      <c r="G58" s="13">
         <v>509.71</v>
       </c>
-      <c r="H58" s="12">
+      <c r="H58" s="11">
         <v>74</v>
       </c>
       <c r="I58">
@@ -3959,10 +3998,10 @@
       <c r="J58">
         <v>35.60859</v>
       </c>
-      <c r="K58" s="14">
+      <c r="K58" s="13">
         <v>1102.07</v>
       </c>
-      <c r="L58" s="12">
+      <c r="L58" s="11">
         <v>100</v>
       </c>
       <c r="M58">
@@ -3971,7 +4010,7 @@
       <c r="N58">
         <v>6.1022999999999996</v>
       </c>
-      <c r="O58" s="14">
+      <c r="O58" s="13">
         <v>210.24</v>
       </c>
       <c r="P58">
@@ -3983,18 +4022,18 @@
       <c r="R58">
         <v>12.711740000000001</v>
       </c>
-      <c r="S58" s="14">
+      <c r="S58" s="13">
         <v>217.77</v>
       </c>
     </row>
     <row r="59" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B59" s="19">
+      <c r="B59" s="18">
         <v>5</v>
       </c>
-      <c r="C59" s="13" t="s">
+      <c r="C59" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="D59" s="12">
+      <c r="D59" s="11">
         <v>53</v>
       </c>
       <c r="E59">
@@ -4003,10 +4042,10 @@
       <c r="F59">
         <v>25.480720000000002</v>
       </c>
-      <c r="G59" s="14">
+      <c r="G59" s="13">
         <v>654.26</v>
       </c>
-      <c r="H59" s="12">
+      <c r="H59" s="11">
         <v>77</v>
       </c>
       <c r="I59">
@@ -4015,10 +4054,10 @@
       <c r="J59">
         <v>28.860240000000001</v>
       </c>
-      <c r="K59" s="14">
+      <c r="K59" s="13">
         <v>695.99</v>
       </c>
-      <c r="L59" s="12">
+      <c r="L59" s="11">
         <v>99</v>
       </c>
       <c r="M59">
@@ -4027,7 +4066,7 @@
       <c r="N59">
         <v>9.1823200000000007</v>
       </c>
-      <c r="O59" s="14">
+      <c r="O59" s="13">
         <v>255.22</v>
       </c>
       <c r="P59">
@@ -4039,18 +4078,18 @@
       <c r="R59">
         <v>12.96635</v>
       </c>
-      <c r="S59" s="14">
+      <c r="S59" s="13">
         <v>147.47999999999999</v>
       </c>
     </row>
     <row r="60" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B60" s="19">
+      <c r="B60" s="18">
         <v>5</v>
       </c>
-      <c r="C60" s="13" t="s">
+      <c r="C60" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="D60" s="12">
+      <c r="D60" s="11">
         <v>56</v>
       </c>
       <c r="E60">
@@ -4059,10 +4098,10 @@
       <c r="F60">
         <v>25.653600000000001</v>
       </c>
-      <c r="G60" s="14">
+      <c r="G60" s="13">
         <v>580.82000000000005</v>
       </c>
-      <c r="H60" s="12">
+      <c r="H60" s="11">
         <v>73</v>
       </c>
       <c r="I60">
@@ -4071,10 +4110,10 @@
       <c r="J60">
         <v>30.77647</v>
       </c>
-      <c r="K60" s="14">
+      <c r="K60" s="13">
         <v>687.32</v>
       </c>
-      <c r="L60" s="12">
+      <c r="L60" s="11">
         <v>95</v>
       </c>
       <c r="M60">
@@ -4083,7 +4122,7 @@
       <c r="N60">
         <v>11.65457</v>
       </c>
-      <c r="O60" s="14">
+      <c r="O60" s="13">
         <v>249.9</v>
       </c>
       <c r="P60">
@@ -4095,18 +4134,18 @@
       <c r="R60">
         <v>9.9598399999999998</v>
       </c>
-      <c r="S60" s="14">
+      <c r="S60" s="13">
         <v>149.04</v>
       </c>
     </row>
     <row r="61" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="19">
+      <c r="B61" s="18">
         <v>5</v>
       </c>
-      <c r="C61" s="13" t="s">
+      <c r="C61" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="D61" s="12">
+      <c r="D61" s="11">
         <v>58</v>
       </c>
       <c r="E61">
@@ -4115,10 +4154,10 @@
       <c r="F61">
         <v>22.591919999999998</v>
       </c>
-      <c r="G61" s="14">
+      <c r="G61" s="13">
         <v>397.21</v>
       </c>
-      <c r="H61" s="12">
+      <c r="H61" s="11">
         <v>93</v>
       </c>
       <c r="I61">
@@ -4127,10 +4166,10 @@
       <c r="J61">
         <v>24.064499999999999</v>
       </c>
-      <c r="K61" s="14">
+      <c r="K61" s="13">
         <v>622.08000000000004</v>
       </c>
-      <c r="L61" s="12">
+      <c r="L61" s="11">
         <v>95</v>
       </c>
       <c r="M61">
@@ -4139,7 +4178,7 @@
       <c r="N61">
         <v>11.27468</v>
       </c>
-      <c r="O61" s="14">
+      <c r="O61" s="13">
         <v>229.58</v>
       </c>
       <c r="P61">
@@ -4151,18 +4190,18 @@
       <c r="R61">
         <v>23.552990000000001</v>
       </c>
-      <c r="S61" s="14">
+      <c r="S61" s="13">
         <v>440.96</v>
       </c>
     </row>
     <row r="62" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B62" s="19">
+      <c r="B62" s="18">
         <v>5</v>
       </c>
-      <c r="C62" s="13" t="s">
+      <c r="C62" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="D62" s="12">
+      <c r="D62" s="11">
         <v>62</v>
       </c>
       <c r="E62">
@@ -4171,10 +4210,10 @@
       <c r="F62">
         <v>28.532250000000001</v>
       </c>
-      <c r="G62" s="14">
+      <c r="G62" s="13">
         <v>613.6</v>
       </c>
-      <c r="H62" s="12">
+      <c r="H62" s="11">
         <v>96</v>
       </c>
       <c r="I62">
@@ -4183,10 +4222,10 @@
       <c r="J62">
         <v>30.581140000000001</v>
       </c>
-      <c r="K62" s="14">
+      <c r="K62" s="13">
         <v>789.59</v>
       </c>
-      <c r="L62" s="12">
+      <c r="L62" s="11">
         <v>95</v>
       </c>
       <c r="M62">
@@ -4195,7 +4234,7 @@
       <c r="N62">
         <v>18.547450000000001</v>
       </c>
-      <c r="O62" s="14">
+      <c r="O62" s="13">
         <v>290.27</v>
       </c>
       <c r="P62">
@@ -4207,63 +4246,63 @@
       <c r="R62">
         <v>7.4397000000000002</v>
       </c>
-      <c r="S62" s="14">
+      <c r="S62" s="13">
         <v>161.61000000000001</v>
       </c>
     </row>
     <row r="63" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B63" s="21">
+      <c r="B63" s="20">
         <v>5</v>
       </c>
-      <c r="C63" s="3" t="s">
+      <c r="C63" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D63" s="15">
+      <c r="D63" s="14">
         <v>62</v>
       </c>
-      <c r="E63" s="16">
+      <c r="E63" s="15">
         <v>25.74896</v>
       </c>
-      <c r="F63" s="16">
+      <c r="F63" s="15">
         <v>25.33174</v>
       </c>
-      <c r="G63" s="17">
+      <c r="G63" s="16">
         <v>408.58</v>
       </c>
-      <c r="H63" s="15">
+      <c r="H63" s="14">
         <v>92</v>
       </c>
-      <c r="I63" s="16">
+      <c r="I63" s="15">
         <v>34.028770000000002</v>
       </c>
-      <c r="J63" s="16">
+      <c r="J63" s="15">
         <v>26.432580000000002</v>
       </c>
-      <c r="K63" s="17">
+      <c r="K63" s="16">
         <v>719.61</v>
       </c>
-      <c r="L63" s="15">
+      <c r="L63" s="14">
         <v>96</v>
       </c>
-      <c r="M63" s="16">
+      <c r="M63" s="15">
         <v>4.0332400000000002</v>
       </c>
-      <c r="N63" s="16">
+      <c r="N63" s="15">
         <v>11.450670000000001</v>
       </c>
-      <c r="O63" s="17">
+      <c r="O63" s="16">
         <v>188.88</v>
       </c>
-      <c r="P63" s="16">
+      <c r="P63" s="15">
         <v>97</v>
       </c>
-      <c r="Q63" s="16">
+      <c r="Q63" s="15">
         <v>5.11334</v>
       </c>
-      <c r="R63" s="16">
+      <c r="R63" s="15">
         <v>8.8681400000000004</v>
       </c>
-      <c r="S63" s="17">
+      <c r="S63" s="16">
         <v>207.58</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update solver logic and webapp components
</commit_message>
<xml_diff>
--- a/results/conference_results.xlsx
+++ b/results/conference_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Thesis\Progress\Original Repo\Multi swarm\ACS-SA-RING\MT-ACS-RING\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1500142-EE63-478A-B203-83AFE3EE5E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BFE775D-3ADD-4B61-AFF9-81A1E8D8F63F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{0FB7F815-C557-4D5B-A7D0-2D04B3DEB5B3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0FB7F815-C557-4D5B-A7D0-2D04B3DEB5B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="50">
   <si>
     <t>Size</t>
   </si>
@@ -455,6 +455,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -477,18 +489,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -833,40 +833,40 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="27" t="s">
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="28" t="s">
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="M2" s="28"/>
-      <c r="N2" s="28"/>
-      <c r="O2" s="28"/>
-      <c r="P2" s="21" t="s">
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="Q2" s="21"/>
-      <c r="R2" s="21"/>
-      <c r="S2" s="21"/>
+      <c r="Q2" s="25"/>
+      <c r="R2" s="25"/>
+      <c r="S2" s="25"/>
     </row>
     <row r="3" spans="2:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="B3" s="23"/>
-      <c r="C3" s="25"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="29"/>
       <c r="D3" s="4" t="s">
         <v>5</v>
       </c>
@@ -920,7 +920,7 @@
       <c r="B4" s="8">
         <v>3</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="8">
@@ -971,15 +971,13 @@
       <c r="S4" s="10">
         <v>25.32</v>
       </c>
-      <c r="U4" s="1" t="s">
-        <v>9</v>
-      </c>
+      <c r="U4" s="1"/>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B5" s="11">
         <v>3</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="22" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="11">
@@ -1030,15 +1028,13 @@
       <c r="S5" s="13">
         <v>33.119999999999997</v>
       </c>
-      <c r="U5" s="12" t="s">
-        <v>10</v>
-      </c>
+      <c r="U5" s="12"/>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B6" s="11">
         <v>3</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="22" t="s">
         <v>11</v>
       </c>
       <c r="D6" s="11">
@@ -1089,15 +1085,13 @@
       <c r="S6" s="13">
         <v>70.849999999999994</v>
       </c>
-      <c r="U6" s="12" t="s">
-        <v>11</v>
-      </c>
+      <c r="U6" s="12"/>
     </row>
     <row r="7" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B7" s="11">
         <v>3</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="22" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="11">
@@ -1148,15 +1142,13 @@
       <c r="S7" s="13">
         <v>35.19</v>
       </c>
-      <c r="U7" s="12" t="s">
-        <v>12</v>
-      </c>
+      <c r="U7" s="12"/>
     </row>
     <row r="8" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B8" s="11">
         <v>3</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="22" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="11">
@@ -1207,15 +1199,13 @@
       <c r="S8" s="13">
         <v>29.21</v>
       </c>
-      <c r="U8" s="12" t="s">
-        <v>13</v>
-      </c>
+      <c r="U8" s="12"/>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B9" s="11">
         <v>3</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="22" t="s">
         <v>14</v>
       </c>
       <c r="D9" s="11">
@@ -1266,15 +1256,13 @@
       <c r="S9" s="13">
         <v>33.07</v>
       </c>
-      <c r="U9" s="12" t="s">
-        <v>14</v>
-      </c>
+      <c r="U9" s="12"/>
     </row>
     <row r="10" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B10" s="11">
         <v>3</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="C10" s="22" t="s">
         <v>15</v>
       </c>
       <c r="D10" s="11">
@@ -1325,15 +1313,13 @@
       <c r="S10" s="13">
         <v>33.200000000000003</v>
       </c>
-      <c r="U10" s="12" t="s">
-        <v>15</v>
-      </c>
+      <c r="U10" s="12"/>
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B11" s="11">
         <v>3</v>
       </c>
-      <c r="C11" s="30" t="s">
+      <c r="C11" s="22" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="11">
@@ -1384,15 +1370,13 @@
       <c r="S11" s="13">
         <v>17.760000000000002</v>
       </c>
-      <c r="U11" s="12" t="s">
-        <v>16</v>
-      </c>
+      <c r="U11" s="12"/>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B12" s="11">
         <v>3</v>
       </c>
-      <c r="C12" s="30" t="s">
+      <c r="C12" s="22" t="s">
         <v>17</v>
       </c>
       <c r="D12" s="11">
@@ -1443,15 +1427,13 @@
       <c r="S12" s="13">
         <v>49.07</v>
       </c>
-      <c r="U12" s="12" t="s">
-        <v>17</v>
-      </c>
+      <c r="U12" s="12"/>
     </row>
     <row r="13" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B13" s="11">
         <v>3</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D13" s="11">
@@ -1502,9 +1484,7 @@
       <c r="S13" s="13">
         <v>34.630000000000003</v>
       </c>
-      <c r="U13" s="12" t="s">
-        <v>18</v>
-      </c>
+      <c r="U13" s="12"/>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B14" s="11">
@@ -2070,7 +2050,7 @@
       <c r="B24" s="17">
         <v>4</v>
       </c>
-      <c r="C24" s="31">
+      <c r="C24" s="23">
         <v>2454</v>
       </c>
       <c r="D24" s="8">
@@ -2126,7 +2106,7 @@
       <c r="B25" s="18">
         <v>4</v>
       </c>
-      <c r="C25" s="32">
+      <c r="C25" s="24">
         <v>2390</v>
       </c>
       <c r="D25" s="11">
@@ -2182,7 +2162,7 @@
       <c r="B26" s="18">
         <v>4</v>
       </c>
-      <c r="C26" s="32">
+      <c r="C26" s="24">
         <v>2357</v>
       </c>
       <c r="D26" s="11">
@@ -2238,7 +2218,7 @@
       <c r="B27" s="18">
         <v>4</v>
       </c>
-      <c r="C27" s="32">
+      <c r="C27" s="24">
         <v>2350</v>
       </c>
       <c r="D27" s="11">
@@ -2294,7 +2274,7 @@
       <c r="B28" s="18">
         <v>4</v>
       </c>
-      <c r="C28" s="32">
+      <c r="C28" s="24">
         <v>2563</v>
       </c>
       <c r="D28" s="11">
@@ -2350,7 +2330,7 @@
       <c r="B29" s="18">
         <v>4</v>
       </c>
-      <c r="C29" s="32">
+      <c r="C29" s="24">
         <v>2456</v>
       </c>
       <c r="D29" s="11">
@@ -2406,7 +2386,7 @@
       <c r="B30" s="18">
         <v>4</v>
       </c>
-      <c r="C30" s="32">
+      <c r="C30" s="24">
         <v>2525</v>
       </c>
       <c r="D30" s="11">
@@ -2462,7 +2442,7 @@
       <c r="B31" s="18">
         <v>4</v>
       </c>
-      <c r="C31" s="32">
+      <c r="C31" s="24">
         <v>2405</v>
       </c>
       <c r="D31" s="11">
@@ -2518,7 +2498,7 @@
       <c r="B32" s="18">
         <v>4</v>
       </c>
-      <c r="C32" s="32">
+      <c r="C32" s="24">
         <v>2281</v>
       </c>
       <c r="D32" s="11">
@@ -2574,7 +2554,7 @@
       <c r="B33" s="18">
         <v>4</v>
       </c>
-      <c r="C33" s="32">
+      <c r="C33" s="24">
         <v>2862</v>
       </c>
       <c r="D33" s="11">
@@ -3190,7 +3170,7 @@
       <c r="B44" s="17">
         <v>5</v>
       </c>
-      <c r="C44" s="29" t="s">
+      <c r="C44" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D44" s="8">
@@ -3246,7 +3226,7 @@
       <c r="B45" s="18">
         <v>5</v>
       </c>
-      <c r="C45" s="30" t="s">
+      <c r="C45" s="22" t="s">
         <v>30</v>
       </c>
       <c r="D45" s="11">
@@ -3302,7 +3282,7 @@
       <c r="B46" s="18">
         <v>5</v>
       </c>
-      <c r="C46" s="30" t="s">
+      <c r="C46" s="22" t="s">
         <v>31</v>
       </c>
       <c r="D46" s="11">
@@ -3358,7 +3338,7 @@
       <c r="B47" s="18">
         <v>5</v>
       </c>
-      <c r="C47" s="30" t="s">
+      <c r="C47" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D47" s="11">
@@ -3414,7 +3394,7 @@
       <c r="B48" s="18">
         <v>5</v>
       </c>
-      <c r="C48" s="30" t="s">
+      <c r="C48" s="22" t="s">
         <v>33</v>
       </c>
       <c r="D48" s="11">
@@ -3470,7 +3450,7 @@
       <c r="B49" s="18">
         <v>5</v>
       </c>
-      <c r="C49" s="30" t="s">
+      <c r="C49" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D49" s="11">
@@ -3526,7 +3506,7 @@
       <c r="B50" s="18">
         <v>5</v>
       </c>
-      <c r="C50" s="30" t="s">
+      <c r="C50" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D50" s="11">
@@ -3582,7 +3562,7 @@
       <c r="B51" s="18">
         <v>5</v>
       </c>
-      <c r="C51" s="30" t="s">
+      <c r="C51" s="22" t="s">
         <v>36</v>
       </c>
       <c r="D51" s="11">
@@ -3638,7 +3618,7 @@
       <c r="B52" s="18">
         <v>5</v>
       </c>
-      <c r="C52" s="30" t="s">
+      <c r="C52" s="22" t="s">
         <v>37</v>
       </c>
       <c r="D52" s="11">
@@ -3694,7 +3674,7 @@
       <c r="B53" s="18">
         <v>5</v>
       </c>
-      <c r="C53" s="30" t="s">
+      <c r="C53" s="22" t="s">
         <v>38</v>
       </c>
       <c r="D53" s="11">

</xml_diff>